<commit_message>
Add v0.6 measurement-ready performance surfaces
</commit_message>
<xml_diff>
--- a/paper/results-workbook.xlsx
+++ b/paper/results-workbook.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9119dc37922d4544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reproduction" sheetId="2" r:id="R2f3a7d7870cc4574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hourly Preview" sheetId="3" r:id="R8be557af7594463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Preview" sheetId="4" r:id="Rec261194eb934129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R0fea66a4947f42bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9e6e6877a0e74c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reproduction" sheetId="2" r:id="R31944f7202184b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hourly Preview" sheetId="3" r:id="R815cd1a25fab476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Preview" sheetId="4" r:id="R8e868714880a4e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rb805fce2e1e0451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurement Demo" sheetId="6" r:id="R7f201f540ac44023"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0.00E+00"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="0.000000"/>
     <x:numFmt numFmtId="203" formatCode="0.000"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.0"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -46,12 +48,32 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4E5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4E5"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -70,7 +92,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -84,6 +106,30 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -388,6 +434,7 @@
     <c:plotArea>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -568,6 +615,118 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Synthetic operational GHG demonstration</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Operational GHG</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Measurement Demo'!$L$2:$L$3</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Measurement Demo'!$M$2:$M$3</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -594,7 +753,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R404aff75f73f481c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R55d79640bdb04095"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -629,7 +788,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R36abf5c56eba4061"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R54c5a30658d44fff"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -664,7 +823,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R01a179c5308a405f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R16e2be2807b44fd2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -673,9 +832,63 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5320c73d748044e0"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:person displayName="Han Hu" id="{51625546-762B-418A-A914-209D94FC9153}"/>
+  <xltc:person displayName="Han Hu" id="{3AD867B9-7451-4915-ADB8-23C704A5ADF9}"/>
+  <xltc:person displayName="Han Hu" id="{AC61255E-CDF8-4624-8A45-3E16F716337B}"/>
 </xltc:personList>
 </file>
 
@@ -874,7 +1087,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
@@ -892,7 +1105,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>OpenDC-LCA v0.4-v0.5 paper results</x:v>
+        <x:v>OpenDC-LCA v0.4-v0.6 paper results</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -1035,13 +1248,53 @@
       <x:c r="D17" s="8"/>
       <x:c r="E17" s="8"/>
     </x:row>
+    <x:row r="19" ht="26" customHeight="1">
+      <x:c r="A19" s="21" t="str">
+        <x:v>v0.6 measurement gate</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>Load-temperature surface</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>Hourly workload integration</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Extrapolation</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Comparative claim</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Blocked for synthetic data</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A15:E17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa51d9f435f04e51"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9e86d3016747e8"/>
 </x:worksheet>
 </file>
 
@@ -2008,7 +2261,7 @@
     <x:mergeCell ref="A7:G10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62fcb234e3204ef5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad74fb4aeca6480e"/>
 </x:worksheet>
 </file>
 
@@ -2582,7 +2835,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9729bf43b6e541e6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf1d5c4955884529"/>
 </x:worksheet>
 </file>
 
@@ -2669,4 +2922,249 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="20" t="str">
+        <x:v>v0.6 measurement-surface protocol demonstration</x:v>
+      </x:c>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
+      <x:c r="L1" t="str">
+        <x:v>Architecture</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>Operational GHG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="L2" t="str">
+        <x:v>air-cooled</x:v>
+      </x:c>
+      <x:c r="M2" t="n">
+        <x:v>486.04382369177256</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="21" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+      <x:c r="B3" s="21" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>direct-to-chip</x:v>
+      </x:c>
+      <x:c r="M3" t="n">
+        <x:v>471.2536294845416</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Evidence status</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>synthetic protocol demonstration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Comparative claim allowed</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Grid factor (kg CO2e/MWh)</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>452.8805904</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="21" t="str">
+        <x:v>Architecture</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>Hours</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>IT energy (kWh)</x:v>
+      </x:c>
+      <x:c r="D8" s="21" t="str">
+        <x:v>Cooling energy (kWh)</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="str">
+        <x:v>On-site water (L)</x:v>
+      </x:c>
+      <x:c r="F8" s="21" t="str">
+        <x:v>Mean PUE</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="str">
+        <x:v>PUE lower</x:v>
+      </x:c>
+      <x:c r="H8" s="21" t="str">
+        <x:v>PUE upper</x:v>
+      </x:c>
+      <x:c r="I8" s="21" t="str">
+        <x:v>Operational kg CO2e/IT MWh</x:v>
+      </x:c>
+      <x:c r="J8" s="21" t="str">
+        <x:v>Evidence status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>air-cooled</x:v>
+      </x:c>
+      <x:c r="B9" s="15" t="n">
+        <x:v>8760</x:v>
+      </x:c>
+      <x:c r="C9" s="15" t="n">
+        <x:v>646050</x:v>
+      </x:c>
+      <x:c r="D9" s="15" t="n">
+        <x:v>47308.51205000029</x:v>
+      </x:c>
+      <x:c r="E9" s="15" t="n">
+        <x:v>8137.7916750000295</x:v>
+      </x:c>
+      <x:c r="F9" s="10" t="n">
+        <x:v>1.073227323040013</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="n">
+        <x:v>1.0695659568880125</x:v>
+      </x:c>
+      <x:c r="H9" s="10" t="n">
+        <x:v>1.0768886891920133</x:v>
+      </x:c>
+      <x:c r="I9" s="10" t="n">
+        <x:v>486.04382369177256</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>synthetic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>direct-to-chip</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="n">
+        <x:v>8760</x:v>
+      </x:c>
+      <x:c r="C10" s="15" t="n">
+        <x:v>646050</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="n">
+        <x:v>26209.782782000362</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="n">
+        <x:v>2170.077779999993</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="n">
+        <x:v>1.040569279130099</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="n">
+        <x:v>1.0385408151735935</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="n">
+        <x:v>1.0425977430866027</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="n">
+        <x:v>471.2536294845416</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>synthetic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="24" t="str">
+        <x:v>Synthetic protocol demonstration only. Bilinear interpolation is restricted to the measured load-temperature envelope. Replace both synthetic maps with reviewed NED3 measurements before making comparative claims.</x:v>
+      </x:c>
+      <x:c r="B12" s="24"/>
+      <x:c r="C12" s="24"/>
+      <x:c r="D12" s="24"/>
+      <x:c r="E12" s="24"/>
+      <x:c r="F12" s="24"/>
+      <x:c r="G12" s="24"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="24"/>
+      <x:c r="J12" s="24"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="24"/>
+      <x:c r="B13" s="24"/>
+      <x:c r="C13" s="24"/>
+      <x:c r="D13" s="24"/>
+      <x:c r="E13" s="24"/>
+      <x:c r="F13" s="24"/>
+      <x:c r="G13" s="24"/>
+      <x:c r="H13" s="24"/>
+      <x:c r="I13" s="24"/>
+      <x:c r="J13" s="24"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="24"/>
+      <x:c r="B14" s="24"/>
+      <x:c r="C14" s="24"/>
+      <x:c r="D14" s="24"/>
+      <x:c r="E14" s="24"/>
+      <x:c r="F14" s="24"/>
+      <x:c r="G14" s="24"/>
+      <x:c r="H14" s="24"/>
+      <x:c r="I14" s="24"/>
+      <x:c r="J14" s="24"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="24"/>
+      <x:c r="B15" s="24"/>
+      <x:c r="C15" s="24"/>
+      <x:c r="D15" s="24"/>
+      <x:c r="E15" s="24"/>
+      <x:c r="F15" s="24"/>
+      <x:c r="G15" s="24"/>
+      <x:c r="H15" s="24"/>
+      <x:c r="I15" s="24"/>
+      <x:c r="J15" s="24"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A12:J15"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b328f2129b44197"/>
+</x:worksheet>
 </file>
</xml_diff>